<commit_message>
Actualización de documentos, considerando cambios realizados en Google Drive
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/1.5 RACI/Matriz RACI.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/1.5 RACI/Matriz RACI.xlsx
@@ -15,28 +15,25 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="39">
   <si>
-    <t>Indicativo</t>
+    <t>Cargo</t>
   </si>
   <si>
-    <t>Cargo</t>
+    <t>Indicativo</t>
   </si>
   <si>
     <t>Actividad / Entregable</t>
   </si>
   <si>
+    <t>Jefe de Proyecto</t>
+  </si>
+  <si>
     <t>Sinificadio</t>
   </si>
   <si>
-    <t>Responsable</t>
+    <t>Especialista en Base de Datos</t>
   </si>
   <si>
-    <t>R</t>
-  </si>
-  <si>
-    <t>Jefe de Proyecto</t>
-  </si>
-  <si>
-    <t>Especialista en Base de Datos</t>
+    <t>Responsable</t>
   </si>
   <si>
     <t>Especialista en Programación Web</t>
@@ -45,10 +42,10 @@
     <t>Especialista en Programación Móvil</t>
   </si>
   <si>
-    <t>Gabriel Valencia</t>
+    <t>Especialista en Metodologías y Documentación</t>
   </si>
   <si>
-    <t>Especialista en Metodologías y Documentación</t>
+    <t>R</t>
   </si>
   <si>
     <t xml:space="preserve"> Especialista en Programación de Escritorio</t>
@@ -57,16 +54,10 @@
     <t>Especialista en QA y Automatización</t>
   </si>
   <si>
-    <t>Alonso Gonzalez</t>
-  </si>
-  <si>
     <t>Especialista en programación FullStack</t>
   </si>
   <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>Aprobador</t>
+    <t>Gabriel Valencia</t>
   </si>
   <si>
     <t>Especialista en Arquitectura de Software</t>
@@ -75,31 +66,40 @@
     <t>Product Owner</t>
   </si>
   <si>
+    <t>Alonso Gonzalez</t>
+  </si>
+  <si>
+    <t>Documentación Inicial, Definición del Proyecto y Metodología</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Gabriel Valencia / Diego Plaza</t>
+  </si>
+  <si>
     <t>C</t>
+  </si>
+  <si>
+    <t>Aprobador</t>
+  </si>
+  <si>
+    <t>Diego Plaza</t>
   </si>
   <si>
     <t>Consultado</t>
   </si>
   <si>
-    <t>Gabriel Valencia / Diego Plaza</t>
-  </si>
-  <si>
-    <t>Documentación Inicial, Definición del Proyecto y Metodología</t>
-  </si>
-  <si>
     <t>I</t>
   </si>
   <si>
-    <t>Informado</t>
-  </si>
-  <si>
-    <t>Diego Plaza</t>
+    <t>Definición de Requisitos Funcionales/No Funcionales</t>
   </si>
   <si>
     <t>Julio Tapia</t>
   </si>
   <si>
-    <t>Definición de Requisitos Funcionales/No Funcionales</t>
+    <t>Informado</t>
   </si>
   <si>
     <t>Planificación de Sprints</t>
@@ -144,6 +144,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="9.0"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="10.0"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -151,13 +158,6 @@
     </font>
     <font>
       <b/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -217,23 +217,23 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -296,12 +296,6 @@
     </dxf>
   </dxfs>
   <tableStyles count="3">
-    <tableStyle count="4" pivot="0" name="Responsable-style">
-      <tableStyleElement dxfId="1" type="headerRow"/>
-      <tableStyleElement dxfId="2" type="firstRowStripe"/>
-      <tableStyleElement dxfId="3" type="secondRowStripe"/>
-      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
-    </tableStyle>
     <tableStyle count="4" pivot="0" name="Leyenda-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
@@ -309,6 +303,12 @@
       <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
     </tableStyle>
     <tableStyle count="4" pivot="0" name="RACI-style">
+      <tableStyleElement dxfId="1" type="headerRow"/>
+      <tableStyleElement dxfId="2" type="firstRowStripe"/>
+      <tableStyleElement dxfId="3" type="secondRowStripe"/>
+      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    </tableStyle>
+    <tableStyle count="4" pivot="0" name="Responsable-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
@@ -580,38 +580,38 @@
   </cols>
   <sheetData>
     <row r="1" ht="92.25" customHeight="1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>6</v>
+      <c r="B1" s="1" t="s">
+        <v>3</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="I1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="J1" s="3" t="s">
-        <v>18</v>
-      </c>
       <c r="K1" s="6" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="L1" s="7"/>
       <c r="M1" s="7"/>
@@ -631,37 +631,37 @@
     </row>
     <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="8" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>16</v>
+      <c r="B2" s="5" t="s">
+        <v>19</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>20</v>
+      <c r="C2" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>20</v>
+      <c r="D2" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>20</v>
+      <c r="E2" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="F2" s="4" t="s">
-        <v>5</v>
+      <c r="F2" s="5" t="s">
+        <v>10</v>
       </c>
-      <c r="G2" s="4" t="s">
-        <v>20</v>
+      <c r="G2" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="H2" s="4" t="s">
-        <v>20</v>
+      <c r="H2" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="I2" s="4" t="s">
-        <v>20</v>
+      <c r="I2" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="J2" s="4" t="s">
-        <v>20</v>
+      <c r="J2" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="K2" s="4" t="s">
-        <v>24</v>
+      <c r="K2" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="N2" s="7"/>
       <c r="O2" s="7"/>
@@ -679,37 +679,37 @@
     </row>
     <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="8" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>16</v>
+      <c r="B3" s="5" t="s">
+        <v>19</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>20</v>
+      <c r="C3" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>20</v>
+      <c r="D3" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="E3" s="4" t="s">
-        <v>20</v>
+      <c r="E3" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="F3" s="4" t="s">
-        <v>5</v>
+      <c r="F3" s="5" t="s">
+        <v>10</v>
       </c>
-      <c r="G3" s="4" t="s">
-        <v>20</v>
+      <c r="G3" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="H3" s="4" t="s">
-        <v>20</v>
+      <c r="H3" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="I3" s="4" t="s">
-        <v>20</v>
+      <c r="I3" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="J3" s="4" t="s">
-        <v>20</v>
+      <c r="J3" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="K3" s="4" t="s">
-        <v>24</v>
+      <c r="K3" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="N3" s="7"/>
       <c r="O3" s="7"/>
@@ -729,35 +729,35 @@
       <c r="A4" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>16</v>
+      <c r="B4" s="5" t="s">
+        <v>19</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>24</v>
+      <c r="C4" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>24</v>
+      <c r="D4" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>24</v>
+      <c r="E4" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="F4" s="4" t="s">
-        <v>5</v>
+      <c r="F4" s="5" t="s">
+        <v>10</v>
       </c>
-      <c r="G4" s="4" t="s">
-        <v>24</v>
+      <c r="G4" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="H4" s="4" t="s">
-        <v>24</v>
+      <c r="H4" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="I4" s="4" t="s">
-        <v>24</v>
+      <c r="I4" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="J4" s="4" t="s">
-        <v>24</v>
+      <c r="J4" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="K4" s="4" t="s">
-        <v>24</v>
+      <c r="K4" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="N4" s="7"/>
       <c r="O4" s="7"/>
@@ -777,35 +777,35 @@
       <c r="A5" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>24</v>
+      <c r="B5" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>20</v>
+      <c r="C5" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>20</v>
+      <c r="D5" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>20</v>
+      <c r="E5" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="F5" s="4" t="s">
-        <v>24</v>
+      <c r="F5" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="G5" s="4" t="s">
-        <v>20</v>
+      <c r="G5" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="H5" s="4" t="s">
-        <v>20</v>
+      <c r="H5" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="I5" s="4" t="s">
-        <v>5</v>
+      <c r="I5" s="5" t="s">
+        <v>10</v>
       </c>
-      <c r="J5" s="4" t="s">
-        <v>16</v>
+      <c r="J5" s="5" t="s">
+        <v>19</v>
       </c>
-      <c r="K5" s="4" t="s">
-        <v>24</v>
+      <c r="K5" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="N5" s="7"/>
       <c r="O5" s="7"/>
@@ -825,35 +825,35 @@
       <c r="A6" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>24</v>
+      <c r="B6" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>20</v>
+      <c r="C6" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>20</v>
+      <c r="D6" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="E6" s="4" t="s">
-        <v>20</v>
+      <c r="E6" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="F6" s="4" t="s">
-        <v>24</v>
+      <c r="F6" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="G6" s="4" t="s">
-        <v>20</v>
+      <c r="G6" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="H6" s="4" t="s">
-        <v>20</v>
+      <c r="H6" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="I6" s="4" t="s">
-        <v>5</v>
+      <c r="I6" s="5" t="s">
+        <v>10</v>
       </c>
-      <c r="J6" s="4" t="s">
-        <v>16</v>
+      <c r="J6" s="5" t="s">
+        <v>19</v>
       </c>
-      <c r="K6" s="4" t="s">
-        <v>24</v>
+      <c r="K6" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="N6" s="7"/>
       <c r="O6" s="7"/>
@@ -873,35 +873,35 @@
       <c r="A7" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>16</v>
+      <c r="B7" s="5" t="s">
+        <v>19</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>5</v>
+      <c r="C7" s="5" t="s">
+        <v>10</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>24</v>
+      <c r="D7" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="E7" s="4" t="s">
-        <v>24</v>
+      <c r="E7" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="F7" s="4" t="s">
-        <v>24</v>
+      <c r="F7" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="G7" s="4" t="s">
-        <v>24</v>
+      <c r="G7" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="H7" s="4" t="s">
-        <v>24</v>
+      <c r="H7" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="I7" s="4" t="s">
-        <v>20</v>
+      <c r="I7" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="J7" s="4" t="s">
-        <v>20</v>
+      <c r="J7" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="K7" s="4" t="s">
-        <v>24</v>
+      <c r="K7" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="L7" s="7"/>
       <c r="M7" s="7"/>
@@ -923,35 +923,35 @@
       <c r="A8" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>24</v>
+      <c r="B8" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>20</v>
+      <c r="C8" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="D8" s="4" t="s">
-        <v>5</v>
+      <c r="D8" s="5" t="s">
+        <v>10</v>
       </c>
-      <c r="E8" s="4" t="s">
-        <v>20</v>
+      <c r="E8" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="F8" s="4" t="s">
-        <v>24</v>
+      <c r="F8" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="G8" s="4" t="s">
-        <v>20</v>
+      <c r="G8" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="H8" s="4" t="s">
-        <v>16</v>
+      <c r="H8" s="5" t="s">
+        <v>19</v>
       </c>
-      <c r="I8" s="4" t="s">
-        <v>20</v>
+      <c r="I8" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="J8" s="4" t="s">
-        <v>24</v>
+      <c r="J8" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="K8" s="4" t="s">
-        <v>24</v>
+      <c r="K8" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="L8" s="7"/>
       <c r="M8" s="7"/>
@@ -973,35 +973,35 @@
       <c r="A9" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>24</v>
+      <c r="B9" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>20</v>
+      <c r="C9" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>20</v>
+      <c r="D9" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="E9" s="4" t="s">
-        <v>5</v>
+      <c r="E9" s="5" t="s">
+        <v>10</v>
       </c>
-      <c r="F9" s="4" t="s">
-        <v>24</v>
+      <c r="F9" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="G9" s="4" t="s">
-        <v>20</v>
+      <c r="G9" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="H9" s="4" t="s">
-        <v>16</v>
+      <c r="H9" s="5" t="s">
+        <v>19</v>
       </c>
-      <c r="I9" s="4" t="s">
-        <v>20</v>
+      <c r="I9" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="J9" s="4" t="s">
-        <v>24</v>
+      <c r="J9" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="K9" s="4" t="s">
-        <v>24</v>
+      <c r="K9" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="L9" s="7"/>
       <c r="M9" s="7"/>
@@ -1023,35 +1023,35 @@
       <c r="A10" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>24</v>
+      <c r="B10" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>20</v>
+      <c r="C10" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>20</v>
+      <c r="D10" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="E10" s="4" t="s">
-        <v>20</v>
+      <c r="E10" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="F10" s="4" t="s">
-        <v>24</v>
+      <c r="F10" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="G10" s="4" t="s">
-        <v>5</v>
+      <c r="G10" s="5" t="s">
+        <v>10</v>
       </c>
-      <c r="H10" s="4" t="s">
-        <v>16</v>
+      <c r="H10" s="5" t="s">
+        <v>19</v>
       </c>
-      <c r="I10" s="4" t="s">
-        <v>20</v>
+      <c r="I10" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="J10" s="4" t="s">
-        <v>24</v>
+      <c r="J10" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="K10" s="4" t="s">
-        <v>24</v>
+      <c r="K10" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="L10" s="7"/>
       <c r="M10" s="7"/>
@@ -1073,35 +1073,35 @@
       <c r="A11" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>16</v>
+      <c r="B11" s="5" t="s">
+        <v>19</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>24</v>
+      <c r="C11" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>24</v>
+      <c r="D11" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="E11" s="4" t="s">
-        <v>24</v>
+      <c r="E11" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="F11" s="4" t="s">
-        <v>20</v>
+      <c r="F11" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="G11" s="4" t="s">
-        <v>24</v>
+      <c r="G11" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="H11" s="4" t="s">
-        <v>5</v>
+      <c r="H11" s="5" t="s">
+        <v>10</v>
       </c>
-      <c r="I11" s="4" t="s">
-        <v>20</v>
+      <c r="I11" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="J11" s="4" t="s">
-        <v>24</v>
+      <c r="J11" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="K11" s="4" t="s">
-        <v>24</v>
+      <c r="K11" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="L11" s="7"/>
       <c r="M11" s="7"/>
@@ -1123,35 +1123,35 @@
       <c r="A12" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>24</v>
+      <c r="B12" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>20</v>
+      <c r="C12" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>20</v>
+      <c r="D12" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="E12" s="4" t="s">
-        <v>20</v>
+      <c r="E12" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="F12" s="4" t="s">
-        <v>24</v>
+      <c r="F12" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="G12" s="4" t="s">
-        <v>20</v>
+      <c r="G12" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="H12" s="4" t="s">
-        <v>16</v>
+      <c r="H12" s="5" t="s">
+        <v>19</v>
       </c>
-      <c r="I12" s="4" t="s">
-        <v>5</v>
+      <c r="I12" s="5" t="s">
+        <v>10</v>
       </c>
-      <c r="J12" s="4" t="s">
-        <v>20</v>
+      <c r="J12" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="K12" s="4" t="s">
-        <v>24</v>
+      <c r="K12" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="L12" s="7"/>
       <c r="M12" s="7"/>
@@ -1173,35 +1173,35 @@
       <c r="A13" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>16</v>
+      <c r="B13" s="5" t="s">
+        <v>19</v>
       </c>
-      <c r="C13" s="4" t="s">
-        <v>20</v>
+      <c r="C13" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>20</v>
+      <c r="D13" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="E13" s="4" t="s">
-        <v>20</v>
+      <c r="E13" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="F13" s="4" t="s">
-        <v>24</v>
+      <c r="F13" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="G13" s="4" t="s">
-        <v>20</v>
+      <c r="G13" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="H13" s="4" t="s">
-        <v>20</v>
+      <c r="H13" s="5" t="s">
+        <v>21</v>
       </c>
-      <c r="I13" s="4" t="s">
-        <v>5</v>
+      <c r="I13" s="5" t="s">
+        <v>10</v>
       </c>
-      <c r="J13" s="4" t="s">
-        <v>24</v>
+      <c r="J13" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="K13" s="4" t="s">
-        <v>24</v>
+      <c r="K13" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="L13" s="7"/>
       <c r="M13" s="7"/>
@@ -28883,90 +28883,90 @@
   </cols>
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
-      <c r="A1" s="2" t="s">
-        <v>1</v>
+      <c r="A1" s="3" t="s">
+        <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="2" ht="22.5" customHeight="1">
-      <c r="A2" s="5" t="s">
+      <c r="B1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>10</v>
+    </row>
+    <row r="2" ht="22.5" customHeight="1">
+      <c r="A2" s="4" t="s">
+        <v>3</v>
       </c>
+      <c r="B2" s="4" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" ht="22.5" customHeight="1">
+      <c r="A4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B4" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" ht="22.5" customHeight="1">
+      <c r="A5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" ht="22.5" customHeight="1">
+      <c r="A6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" ht="22.5" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="5" t="s">
-        <v>8</v>
+    <row r="8" ht="22.5" customHeight="1">
+      <c r="A8" s="4" t="s">
+        <v>12</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" ht="22.5" customHeight="1">
-      <c r="A6" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="5" t="s">
+    <row r="9" ht="22.5" customHeight="1">
+      <c r="A9" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="5" t="s">
-        <v>10</v>
+      <c r="B9" s="4" t="s">
+        <v>23</v>
       </c>
     </row>
-    <row r="9" ht="22.5" customHeight="1">
-      <c r="A9" s="5" t="s">
+    <row r="10" ht="22.5" customHeight="1">
+      <c r="A10" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="5" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" ht="22.5" customHeight="1">
-      <c r="A10" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>26</v>
+      <c r="B10" s="4" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="9" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="4" t="s">
         <v>27</v>
       </c>
     </row>
@@ -28990,43 +28990,43 @@
   </cols>
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
+      <c r="A1" s="2" t="s">
+        <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" ht="22.5" customHeight="1">
-      <c r="A2" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="5" t="s">
+      <c r="B1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
+    <row r="2" ht="22.5" customHeight="1">
+      <c r="A2" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
     <row r="3" ht="22.5" customHeight="1">
-      <c r="A3" s="4" t="s">
-        <v>16</v>
+      <c r="A3" s="5" t="s">
+        <v>19</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>17</v>
+      <c r="B3" s="4" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B4" s="5" t="s">
+      <c r="A4" s="5" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="4" t="s">
+      <c r="B4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="5" t="s">
+    </row>
+    <row r="5" ht="22.5" customHeight="1">
+      <c r="A5" s="5" t="s">
         <v>25</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
actualizar archivos del drive
fueron subidos los documentos del drive
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/1.5 RACI/Matriz RACI.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/1.5 RACI/Matriz RACI.xlsx
@@ -15,28 +15,31 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="39">
   <si>
-    <t>Indicativo</t>
+    <t>Cargo</t>
   </si>
   <si>
-    <t>Cargo</t>
+    <t>Indicativo</t>
   </si>
   <si>
     <t>Actividad / Entregable</t>
   </si>
   <si>
-    <t>Sinificadio</t>
+    <t>Responsable</t>
   </si>
   <si>
-    <t>Responsable</t>
+    <t>Jefe de Proyecto</t>
+  </si>
+  <si>
+    <t>Sinificadio</t>
   </si>
   <si>
     <t>R</t>
   </si>
   <si>
-    <t>Jefe de Proyecto</t>
+    <t>Especialista en Base de Datos</t>
   </si>
   <si>
-    <t>Especialista en Base de Datos</t>
+    <t>Gabriel Valencia</t>
   </si>
   <si>
     <t>Especialista en Programación Web</t>
@@ -45,7 +48,7 @@
     <t>Especialista en Programación Móvil</t>
   </si>
   <si>
-    <t>Gabriel Valencia</t>
+    <t>Alonso Gonzalez</t>
   </si>
   <si>
     <t>Especialista en Metodologías y Documentación</t>
@@ -57,10 +60,19 @@
     <t>Especialista en QA y Automatización</t>
   </si>
   <si>
-    <t>Alonso Gonzalez</t>
+    <t>Especialista en programación FullStack</t>
   </si>
   <si>
-    <t>Especialista en programación FullStack</t>
+    <t>Especialista en Arquitectura de Software</t>
+  </si>
+  <si>
+    <t>Product Owner</t>
+  </si>
+  <si>
+    <t>Gabriel Valencia / Diego Plaza</t>
+  </si>
+  <si>
+    <t>Documentación Inicial, Definición del Proyecto y Metodología</t>
   </si>
   <si>
     <t>A</t>
@@ -69,31 +81,19 @@
     <t>Aprobador</t>
   </si>
   <si>
-    <t>Especialista en Arquitectura de Software</t>
-  </si>
-  <si>
-    <t>Product Owner</t>
-  </si>
-  <si>
     <t>C</t>
   </si>
   <si>
     <t>Consultado</t>
   </si>
   <si>
-    <t>Gabriel Valencia / Diego Plaza</t>
-  </si>
-  <si>
-    <t>Documentación Inicial, Definición del Proyecto y Metodología</t>
+    <t>Diego Plaza</t>
   </si>
   <si>
     <t>I</t>
   </si>
   <si>
     <t>Informado</t>
-  </si>
-  <si>
-    <t>Diego Plaza</t>
   </si>
   <si>
     <t>Julio Tapia</t>
@@ -144,13 +144,13 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10.0"/>
+      <b/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <sz val="10.0"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -217,23 +217,23 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="1" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -302,13 +302,13 @@
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
       <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
     </tableStyle>
-    <tableStyle count="4" pivot="0" name="Leyenda-style">
+    <tableStyle count="4" pivot="0" name="RACI-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
       <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
     </tableStyle>
-    <tableStyle count="4" pivot="0" name="RACI-style">
+    <tableStyle count="4" pivot="0" name="Leyenda-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
@@ -335,7 +335,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:K13" displayName="RACI" name="RACI" id="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:K13" displayName="RACI" name="RACI" id="2">
   <tableColumns count="11">
     <tableColumn name="Actividad / Entregable" id="1"/>
     <tableColumn name="Jefe de Proyecto" id="2"/>
@@ -364,7 +364,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:B5" displayName="Leyenda" name="Leyenda" id="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:B5" displayName="Leyenda" name="Leyenda" id="3">
   <tableColumns count="2">
     <tableColumn name="Indicativo" id="1"/>
     <tableColumn name="Sinificadio" id="2"/>
@@ -584,34 +584,34 @@
         <v>2</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I1" s="3" t="s">
         <v>15</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="L1" s="7"/>
       <c r="M1" s="7"/>
@@ -631,37 +631,37 @@
     </row>
     <row r="2" ht="22.5" customHeight="1">
       <c r="A2" s="8" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="4" t="s">
-        <v>20</v>
+      <c r="C2" s="5" t="s">
+        <v>22</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>20</v>
+      <c r="D2" s="5" t="s">
+        <v>22</v>
       </c>
-      <c r="F2" s="4" t="s">
-        <v>5</v>
+      <c r="E2" s="5" t="s">
+        <v>22</v>
       </c>
-      <c r="G2" s="4" t="s">
-        <v>20</v>
+      <c r="F2" s="5" t="s">
+        <v>6</v>
       </c>
-      <c r="H2" s="4" t="s">
-        <v>20</v>
+      <c r="G2" s="5" t="s">
+        <v>22</v>
       </c>
-      <c r="I2" s="4" t="s">
-        <v>20</v>
+      <c r="H2" s="5" t="s">
+        <v>22</v>
       </c>
-      <c r="J2" s="4" t="s">
-        <v>20</v>
+      <c r="I2" s="5" t="s">
+        <v>22</v>
       </c>
-      <c r="K2" s="4" t="s">
-        <v>24</v>
+      <c r="J2" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="N2" s="7"/>
       <c r="O2" s="7"/>
@@ -681,35 +681,35 @@
       <c r="A3" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>20</v>
+      <c r="C3" s="5" t="s">
+        <v>22</v>
       </c>
-      <c r="E3" s="4" t="s">
-        <v>20</v>
+      <c r="D3" s="5" t="s">
+        <v>22</v>
       </c>
-      <c r="F3" s="4" t="s">
-        <v>5</v>
+      <c r="E3" s="5" t="s">
+        <v>22</v>
       </c>
-      <c r="G3" s="4" t="s">
-        <v>20</v>
+      <c r="F3" s="5" t="s">
+        <v>6</v>
       </c>
-      <c r="H3" s="4" t="s">
-        <v>20</v>
+      <c r="G3" s="5" t="s">
+        <v>22</v>
       </c>
-      <c r="I3" s="4" t="s">
-        <v>20</v>
+      <c r="H3" s="5" t="s">
+        <v>22</v>
       </c>
-      <c r="J3" s="4" t="s">
-        <v>20</v>
+      <c r="I3" s="5" t="s">
+        <v>22</v>
       </c>
-      <c r="K3" s="4" t="s">
-        <v>24</v>
+      <c r="J3" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="N3" s="7"/>
       <c r="O3" s="7"/>
@@ -729,35 +729,35 @@
       <c r="A4" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>16</v>
+      <c r="B4" s="5" t="s">
+        <v>20</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>24</v>
+      <c r="C4" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>24</v>
+      <c r="D4" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>24</v>
+      <c r="E4" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="F4" s="4" t="s">
-        <v>5</v>
+      <c r="F4" s="5" t="s">
+        <v>6</v>
       </c>
-      <c r="G4" s="4" t="s">
-        <v>24</v>
+      <c r="G4" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="H4" s="4" t="s">
-        <v>24</v>
+      <c r="H4" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="I4" s="4" t="s">
-        <v>24</v>
+      <c r="I4" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="J4" s="4" t="s">
-        <v>24</v>
+      <c r="J4" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="K4" s="4" t="s">
-        <v>24</v>
+      <c r="K4" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="N4" s="7"/>
       <c r="O4" s="7"/>
@@ -777,35 +777,35 @@
       <c r="A5" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>24</v>
+      <c r="B5" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="J5" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>24</v>
+      <c r="K5" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="N5" s="7"/>
       <c r="O5" s="7"/>
@@ -825,35 +825,35 @@
       <c r="A6" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="4" t="s">
-        <v>24</v>
+      <c r="B6" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="J6" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="J6" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>24</v>
+      <c r="K6" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="N6" s="7"/>
       <c r="O6" s="7"/>
@@ -873,35 +873,35 @@
       <c r="A7" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="I7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="J7" s="4" t="s">
-        <v>20</v>
+      <c r="C7" s="5" t="s">
+        <v>6</v>
       </c>
-      <c r="K7" s="4" t="s">
-        <v>24</v>
+      <c r="D7" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="L7" s="7"/>
       <c r="M7" s="7"/>
@@ -923,35 +923,35 @@
       <c r="A8" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>24</v>
+      <c r="B8" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H8" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="4" t="s">
-        <v>5</v>
+      <c r="I8" s="5" t="s">
+        <v>22</v>
       </c>
-      <c r="E8" s="4" t="s">
-        <v>20</v>
+      <c r="J8" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="F8" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="K8" s="4" t="s">
-        <v>24</v>
+      <c r="K8" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="L8" s="7"/>
       <c r="M8" s="7"/>
@@ -973,35 +973,35 @@
       <c r="A9" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>24</v>
+      <c r="B9" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H9" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>20</v>
+      <c r="I9" s="5" t="s">
+        <v>22</v>
       </c>
-      <c r="E9" s="4" t="s">
-        <v>5</v>
+      <c r="J9" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="F9" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="J9" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="K9" s="4" t="s">
-        <v>24</v>
+      <c r="K9" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="L9" s="7"/>
       <c r="M9" s="7"/>
@@ -1023,35 +1023,35 @@
       <c r="A10" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>24</v>
+      <c r="B10" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H10" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>20</v>
+      <c r="I10" s="5" t="s">
+        <v>22</v>
       </c>
-      <c r="E10" s="4" t="s">
-        <v>20</v>
+      <c r="J10" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="F10" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="K10" s="4" t="s">
-        <v>24</v>
+      <c r="K10" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="L10" s="7"/>
       <c r="M10" s="7"/>
@@ -1073,35 +1073,35 @@
       <c r="A11" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="G11" s="4" t="s">
-        <v>24</v>
+      <c r="C11" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="H11" s="4" t="s">
-        <v>5</v>
+      <c r="D11" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="I11" s="4" t="s">
-        <v>20</v>
+      <c r="E11" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="J11" s="4" t="s">
-        <v>24</v>
+      <c r="F11" s="5" t="s">
+        <v>22</v>
       </c>
-      <c r="K11" s="4" t="s">
-        <v>24</v>
+      <c r="G11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="L11" s="7"/>
       <c r="M11" s="7"/>
@@ -1123,35 +1123,35 @@
       <c r="A12" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>24</v>
+      <c r="B12" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H12" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>20</v>
+      <c r="I12" s="5" t="s">
+        <v>6</v>
       </c>
-      <c r="E12" s="4" t="s">
-        <v>20</v>
+      <c r="J12" s="5" t="s">
+        <v>22</v>
       </c>
-      <c r="F12" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="J12" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="K12" s="4" t="s">
-        <v>24</v>
+      <c r="K12" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="L12" s="7"/>
       <c r="M12" s="7"/>
@@ -1173,35 +1173,35 @@
       <c r="A13" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>20</v>
+      <c r="C13" s="5" t="s">
+        <v>22</v>
       </c>
-      <c r="E13" s="4" t="s">
-        <v>20</v>
+      <c r="D13" s="5" t="s">
+        <v>22</v>
       </c>
-      <c r="F13" s="4" t="s">
-        <v>24</v>
+      <c r="E13" s="5" t="s">
+        <v>22</v>
       </c>
-      <c r="G13" s="4" t="s">
-        <v>20</v>
+      <c r="F13" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="H13" s="4" t="s">
-        <v>20</v>
+      <c r="G13" s="5" t="s">
+        <v>22</v>
       </c>
-      <c r="I13" s="4" t="s">
-        <v>5</v>
+      <c r="H13" s="5" t="s">
+        <v>22</v>
       </c>
-      <c r="J13" s="4" t="s">
-        <v>24</v>
+      <c r="I13" s="5" t="s">
+        <v>6</v>
       </c>
-      <c r="K13" s="4" t="s">
-        <v>24</v>
+      <c r="J13" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>25</v>
       </c>
       <c r="L13" s="7"/>
       <c r="M13" s="7"/>
@@ -28883,90 +28883,90 @@
   </cols>
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
-      <c r="A1" s="2" t="s">
-        <v>1</v>
+      <c r="A1" s="1" t="s">
+        <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" ht="22.5" customHeight="1">
+      <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" ht="22.5" customHeight="1">
-      <c r="A2" s="5" t="s">
-        <v>6</v>
+      <c r="B2" s="4" t="s">
+        <v>8</v>
       </c>
-      <c r="B2" s="5" t="s">
+    </row>
+    <row r="3" ht="22.5" customHeight="1">
+      <c r="A3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" ht="22.5" customHeight="1">
+      <c r="A4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" ht="22.5" customHeight="1">
+      <c r="A5" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" ht="22.5" customHeight="1">
-      <c r="A3" s="5" t="s">
-        <v>7</v>
+      <c r="B5" s="4" t="s">
+        <v>11</v>
       </c>
-      <c r="B3" s="5" t="s">
+    </row>
+    <row r="6" ht="22.5" customHeight="1">
+      <c r="A6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" ht="22.5" customHeight="1">
+      <c r="A7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" ht="22.5" customHeight="1">
+      <c r="A8" s="4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" ht="22.5" customHeight="1">
-      <c r="A6" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>10</v>
-      </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="5" t="s">
-        <v>26</v>
+      <c r="B9" s="4" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
-      <c r="A10" s="5" t="s">
-        <v>18</v>
+      <c r="A10" s="4" t="s">
+        <v>16</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>26</v>
+      <c r="B10" s="4" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
       <c r="A11" s="9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="4" t="s">
         <v>27</v>
       </c>
     </row>
@@ -28990,43 +28990,43 @@
   </cols>
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
+      <c r="A1" s="2" t="s">
+        <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" ht="22.5" customHeight="1">
+      <c r="A2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" ht="22.5" customHeight="1">
-      <c r="A2" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>4</v>
-      </c>
-    </row>
     <row r="3" ht="22.5" customHeight="1">
-      <c r="A3" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="4" t="s">
+      <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>21</v>
       </c>
     </row>
+    <row r="4" ht="22.5" customHeight="1">
+      <c r="A4" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
     <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="4" t="s">
-        <v>24</v>
+      <c r="A5" s="5" t="s">
+        <v>25</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>25</v>
+      <c r="B5" s="4" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>